<commit_message>
feat: Update email template Excel file
</commit_message>
<xml_diff>
--- a/public/email-sablonu.xlsx
+++ b/public/email-sablonu.xlsx
@@ -1,44 +1,299 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alperbayram/Desktop/GDG/2026/ıwd/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8671DCBC-D189-3844-9C6A-78A8730B7510}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="Katılımcılar" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="81">
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>aleynacif5@gmail.com</t>
+  </si>
+  <si>
+    <t>haticenidapolat@outlook.com</t>
+  </si>
+  <si>
+    <t>esin.fuzz@gmail.com</t>
+  </si>
+  <si>
+    <t>gozdeyldrm188@gmail.com</t>
+  </si>
+  <si>
+    <t>mertenesakarsu@gmail.com</t>
+  </si>
+  <si>
+    <t>snmzpolat@gmail.com</t>
+  </si>
+  <si>
+    <t>elifsuarikan09@gmail.com</t>
+  </si>
+  <si>
+    <t>burhackmutlu@gmail.com</t>
+  </si>
+  <si>
+    <t>canandulgeroglu@gmail.com</t>
+  </si>
+  <si>
+    <t>berrameral.durmaz@std.antalya.edu.tr</t>
+  </si>
+  <si>
+    <t>bfsanli@gmail.com</t>
+  </si>
+  <si>
+    <t>cbcanseribozkus1@gmail.com</t>
+  </si>
+  <si>
+    <t>uluberfinipek@gmail.com</t>
+  </si>
+  <si>
+    <t>incemehmetbilal@gmail.com</t>
+  </si>
+  <si>
+    <t>simge.hatip@gmail.com</t>
+  </si>
+  <si>
+    <t>seda.kader2002@yandex.com</t>
+  </si>
+  <si>
+    <t>yagmur.durmus23@icloud.com</t>
+  </si>
+  <si>
+    <t>e.gulce14@gmail.com</t>
+  </si>
+  <si>
+    <t>halilzeybek.contact@gmail.com</t>
+  </si>
+  <si>
+    <t>simin.mulla@std.antalya.edu.tr</t>
+  </si>
+  <si>
+    <t>z.adaozkan@gmail.com</t>
+  </si>
+  <si>
+    <t>berilss1@outlook.com</t>
+  </si>
+  <si>
+    <t>zorlusemanur0@gmail.com</t>
+  </si>
+  <si>
+    <t>gzdknk@hotmail.com</t>
+  </si>
+  <si>
+    <t>zehrakose207@hotmail.com</t>
+  </si>
+  <si>
+    <t>olmezberfindilara@gmail.com</t>
+  </si>
+  <si>
+    <t>rabiagizemb@gmail.com</t>
+  </si>
+  <si>
+    <t>deryaslhoglu.54@gmail.com</t>
+  </si>
+  <si>
+    <t>a.ozdemir.work@gmail.com</t>
+  </si>
+  <si>
+    <t>fatma.oz315@gmail.com</t>
+  </si>
+  <si>
+    <t>levent1360@gmail.com</t>
+  </si>
+  <si>
+    <t>selinnozlukk@gmail.com</t>
+  </si>
+  <si>
+    <t>alinaisakul2505@gmail.com</t>
+  </si>
+  <si>
+    <t>cetinkalagan1903@gmail.com</t>
+  </si>
+  <si>
+    <t>eminedurues@hotmail.com</t>
+  </si>
+  <si>
+    <t>ulas-koksal@outlook.com.tr</t>
+  </si>
+  <si>
+    <t>saadet.durukan@argeteknoparkmalimusavirlik.com</t>
+  </si>
+  <si>
+    <t>bensuusluu@gmail.com</t>
+  </si>
+  <si>
+    <t>iremyntm19@gmail.com</t>
+  </si>
+  <si>
+    <t>f.eren.ozcelik@gmail.com</t>
+  </si>
+  <si>
+    <t>harun@isikay.com</t>
+  </si>
+  <si>
+    <t>merveffdan@gmail.com</t>
+  </si>
+  <si>
+    <t>sdnr.shn06@gmail.com</t>
+  </si>
+  <si>
+    <t>rumeysa.kisacik@e-vet.com.tr</t>
+  </si>
+  <si>
+    <t>sarpkucuk@gmail.com</t>
+  </si>
+  <si>
+    <t>buse5901@hotmail.com</t>
+  </si>
+  <si>
+    <t>yusufozyazgan@outlook.com</t>
+  </si>
+  <si>
+    <t>omerfarukdasdemir8@gmail.com</t>
+  </si>
+  <si>
+    <t>kbayram038@gmail.com</t>
+  </si>
+  <si>
+    <t>aysegulbulut@gmail.com</t>
+  </si>
+  <si>
+    <t>cetinbeyza28@gmail.com</t>
+  </si>
+  <si>
+    <t>sametarar6607@gmail.com</t>
+  </si>
+  <si>
+    <t>sevvalyntm07@gmail.com</t>
+  </si>
+  <si>
+    <t>kocagozz123@gmail.com</t>
+  </si>
+  <si>
+    <t>ahmetayykan@gmail.com</t>
+  </si>
+  <si>
+    <t>hirasirin81@gmail.com</t>
+  </si>
+  <si>
+    <t>besercagatay@gmail.com</t>
+  </si>
+  <si>
+    <t>toklufatmanur07@gmail.com</t>
+  </si>
+  <si>
+    <t>bilgin.eren923@gmail.com</t>
+  </si>
+  <si>
+    <t>yarenertugrul07@gmail.com</t>
+  </si>
+  <si>
+    <t>alperbayrmm@gmail.com</t>
+  </si>
+  <si>
+    <t>rem1035@hotmail.com</t>
+  </si>
+  <si>
+    <t>yorukarif2008@gmail.com</t>
+  </si>
+  <si>
+    <t>alperensarcayr@gmail.com</t>
+  </si>
+  <si>
+    <t>info@elchedo.pro</t>
+  </si>
+  <si>
+    <t>cc5141864@gmail.com</t>
+  </si>
+  <si>
+    <t>dguk21@gmail.com</t>
+  </si>
+  <si>
+    <t>capkurtdidemsevim@gmail.com</t>
+  </si>
+  <si>
+    <t>dogukanturksoy1999@gmail.com</t>
+  </si>
+  <si>
+    <t>eyuphantilki41@gmail.com</t>
+  </si>
+  <si>
+    <t>kiymazaslanfatma@gmail.com</t>
+  </si>
+  <si>
+    <t>Kirogluhasan08@gmail.com</t>
+  </si>
+  <si>
+    <t>bakicapica@gmail.com</t>
+  </si>
+  <si>
+    <t>ozan.zeray@hotmail.com</t>
+  </si>
+  <si>
+    <t>karaserkan2@gmail.com</t>
+  </si>
+  <si>
+    <t>osmn.ozdmr.07@gmail.com</t>
+  </si>
+  <si>
+    <t>radar1radar1org@gmail.com</t>
+  </si>
+  <si>
+    <t>tolga.yig@gmail.com</t>
+  </si>
+  <si>
+    <t>akinturgut737@gmail.com</t>
+  </si>
+  <si>
+    <t>uakdemir@gmail.com</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -61,17 +316,28 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Köprü" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,32 +662,441 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:A81"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="30.5" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Email</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>ornek1@gmail.com</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>ornek2@gmail.com</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>ornek3@gmail.com</v>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A61" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A62" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A63" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A64" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A65" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A66" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A67" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A68" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A69" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A70" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A71" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A72" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A73" s="1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A74" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A75" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A76" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A77" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A78" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A79" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A80" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A81" s="1" t="s">
+        <v>80</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A65" r:id="rId1" display="mailto:alperensarcayr@gmail.com" xr:uid="{06658918-687B-1347-B675-CC5C5BFCF91F}"/>
+    <hyperlink ref="A66" r:id="rId2" display="mailto:info@elchedo.pro" xr:uid="{F237D509-9129-BE47-A18D-473A1A06207A}"/>
+    <hyperlink ref="A67" r:id="rId3" display="mailto:cc5141864@gmail.com" xr:uid="{61FC5266-8368-DD4F-B177-452C3C0903D8}"/>
+    <hyperlink ref="A68" r:id="rId4" display="mailto:dguk21@gmail.com" xr:uid="{D68F8747-E451-934A-A817-A48D53F72BD5}"/>
+    <hyperlink ref="A69" r:id="rId5" display="mailto:capkurtdidemsevim@gmail.com" xr:uid="{B252AC13-D35C-D042-8AF8-0829EF8FBF9F}"/>
+    <hyperlink ref="A70" r:id="rId6" display="mailto:dogukanturksoy1999@gmail.com" xr:uid="{1E3D7200-4681-BE4D-9064-98D0E903E19C}"/>
+    <hyperlink ref="A71" r:id="rId7" display="mailto:eyuphantilki41@gmail.com" xr:uid="{5643087D-A516-DE4F-B3A1-ABD32096C308}"/>
+    <hyperlink ref="A72" r:id="rId8" display="mailto:kiymazaslanfatma@gmail.com" xr:uid="{39EF22EA-85E5-994E-A5CF-1BF1F5BBFD0F}"/>
+    <hyperlink ref="A73" r:id="rId9" display="mailto:Kirogluhasan08@gmail.com" xr:uid="{7720F11B-F4BF-9945-9159-503646E88A7E}"/>
+    <hyperlink ref="A74" r:id="rId10" display="mailto:bakicapica@gmail.com" xr:uid="{59A7D5F2-AB8E-054F-882C-D7EDCD88EC1B}"/>
+    <hyperlink ref="A75" r:id="rId11" display="mailto:ozan.zeray@hotmail.com" xr:uid="{7B913CB5-A0DF-D244-BB40-392DE02F9CB1}"/>
+    <hyperlink ref="A76" r:id="rId12" display="mailto:karaserkan2@gmail.com" xr:uid="{FFF2B194-E361-5B4C-BA3A-83939AF0DA12}"/>
+    <hyperlink ref="A77" r:id="rId13" display="mailto:osmn.ozdmr.07@gmail.com" xr:uid="{A6775528-8948-2A43-9555-CA6DC1CDBCF4}"/>
+    <hyperlink ref="A78" r:id="rId14" display="mailto:radar1radar1org@gmail.com" xr:uid="{D6211F92-F75A-2A46-A7AC-D74E5729349F}"/>
+    <hyperlink ref="A79" r:id="rId15" display="mailto:tolga.yig@gmail.com" xr:uid="{2F9B8BC4-55E2-3143-88B3-1AF70CBDBAFC}"/>
+    <hyperlink ref="A80" r:id="rId16" display="mailto:akinturgut737@gmail.com" xr:uid="{C12E85A8-AAFC-BC4B-9A36-E112A50C1E3A}"/>
+    <hyperlink ref="A81" r:id="rId17" display="mailto:uakdemir@gmail.com" xr:uid="{2D5C8DA6-04EF-1845-95F5-1894BF31F43D}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A4"/>
+    <ignoredError sqref="A1" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: Update fetch path for email template and add error handling
</commit_message>
<xml_diff>
--- a/public/email-sablonu.xlsx
+++ b/public/email-sablonu.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alperbayram/Desktop/GDG/2026/ıwd/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8671DCBC-D189-3844-9C6A-78A8730B7510}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45E8697A-96D1-9540-93D9-86D0EB169D3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="1120" windowWidth="28800" windowHeight="16020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Katılımcılar" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="85">
   <si>
     <t>Email</t>
   </si>
@@ -221,9 +221,6 @@
     <t>alperbayrmm@gmail.com</t>
   </si>
   <si>
-    <t>rem1035@hotmail.com</t>
-  </si>
-  <si>
     <t>yorukarif2008@gmail.com</t>
   </si>
   <si>
@@ -276,13 +273,28 @@
   </si>
   <si>
     <t>uakdemir@gmail.com</t>
+  </si>
+  <si>
+    <t>gurkan17123@gmail.com</t>
+  </si>
+  <si>
+    <t>omeraksu252525@gmail.com</t>
+  </si>
+  <si>
+    <t>salihayklmz.06@gmail.com</t>
+  </si>
+  <si>
+    <t>emretkszz@gmail.com</t>
+  </si>
+  <si>
+    <t>turkkoyluy@gmail.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -294,6 +306,13 @@
       <u/>
       <sz val="12"/>
       <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -320,9 +339,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Köprü" xfId="1" builtinId="8"/>
@@ -663,10 +683,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A81"/>
+  <dimension ref="A1:A85"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="30.5" customWidth="1"/>
+    <col min="1" max="1" width="51" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
@@ -675,424 +695,444 @@
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+      <c r="A2" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A7" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A8" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A9" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A10" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A11" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A12" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A13" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A14" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A15" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A16" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A17" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A18" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A19" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A20" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A21" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A22" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A23" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A24" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A25" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A26" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A27" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A28" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A29" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A25" t="s">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A30" s="2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A26" t="s">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A31" s="2" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A27" t="s">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A32" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A28" t="s">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A33" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A29" t="s">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A34" s="2" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A30" t="s">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A35" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A31" t="s">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A36" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A32" t="s">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A37" s="2" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A33" t="s">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A38" s="2" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A34" t="s">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A39" s="2" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A35" t="s">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A40" s="2" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A36" t="s">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A41" s="2" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A37" t="s">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A42" s="2" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A38" t="s">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A43" s="2" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A39" t="s">
+    <row r="44" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A44" s="2" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A40" t="s">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A45" s="2" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A41" t="s">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A46" s="2" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A42" t="s">
+    <row r="47" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A47" s="2" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A43" t="s">
+    <row r="48" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A48" s="2" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A44" t="s">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A49" s="2" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A45" t="s">
+    <row r="50" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A50" s="2" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A46" t="s">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A51" s="2" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A47" t="s">
+    <row r="52" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A52" s="2" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A48" t="s">
+    <row r="53" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A53" s="2" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A49" t="s">
+    <row r="54" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A54" s="2" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A50" t="s">
+    <row r="55" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A55" s="2" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A51" t="s">
+    <row r="56" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A56" s="2" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A52" t="s">
+    <row r="57" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A57" s="2" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A53" t="s">
+    <row r="58" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A58" s="2" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A54" t="s">
+    <row r="59" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A59" s="2" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A55" t="s">
+    <row r="60" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A60" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A56" t="s">
+    <row r="61" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A61" s="2" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A57" t="s">
+    <row r="62" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A62" s="2" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A58" t="s">
+    <row r="63" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A63" s="2" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A59" t="s">
+    <row r="64" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A64" s="2" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A60" t="s">
+    <row r="65" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A65" s="2" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A61" t="s">
+    <row r="66" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A66" s="2" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A62" t="s">
+    <row r="67" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A67" s="2" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A63" t="s">
+    <row r="68" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A68" t="s">
         <v>62</v>
-      </c>
-    </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A64" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A65" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A66" s="1" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A67" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A68" s="1" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A69" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A70" s="1" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A71" s="1" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A72" s="1" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A73" s="1" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A74" s="1" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A75" s="1" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A76" s="1" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A77" s="1" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A78" s="1" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A79" s="1" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A80" s="1" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A81" s="1" t="s">
-        <v>80</v>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A82" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A83" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A84" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="85" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A85" s="1" t="s">
+        <v>79</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A65" r:id="rId1" display="mailto:alperensarcayr@gmail.com" xr:uid="{06658918-687B-1347-B675-CC5C5BFCF91F}"/>
-    <hyperlink ref="A66" r:id="rId2" display="mailto:info@elchedo.pro" xr:uid="{F237D509-9129-BE47-A18D-473A1A06207A}"/>
-    <hyperlink ref="A67" r:id="rId3" display="mailto:cc5141864@gmail.com" xr:uid="{61FC5266-8368-DD4F-B177-452C3C0903D8}"/>
-    <hyperlink ref="A68" r:id="rId4" display="mailto:dguk21@gmail.com" xr:uid="{D68F8747-E451-934A-A817-A48D53F72BD5}"/>
-    <hyperlink ref="A69" r:id="rId5" display="mailto:capkurtdidemsevim@gmail.com" xr:uid="{B252AC13-D35C-D042-8AF8-0829EF8FBF9F}"/>
-    <hyperlink ref="A70" r:id="rId6" display="mailto:dogukanturksoy1999@gmail.com" xr:uid="{1E3D7200-4681-BE4D-9064-98D0E903E19C}"/>
-    <hyperlink ref="A71" r:id="rId7" display="mailto:eyuphantilki41@gmail.com" xr:uid="{5643087D-A516-DE4F-B3A1-ABD32096C308}"/>
-    <hyperlink ref="A72" r:id="rId8" display="mailto:kiymazaslanfatma@gmail.com" xr:uid="{39EF22EA-85E5-994E-A5CF-1BF1F5BBFD0F}"/>
-    <hyperlink ref="A73" r:id="rId9" display="mailto:Kirogluhasan08@gmail.com" xr:uid="{7720F11B-F4BF-9945-9159-503646E88A7E}"/>
-    <hyperlink ref="A74" r:id="rId10" display="mailto:bakicapica@gmail.com" xr:uid="{59A7D5F2-AB8E-054F-882C-D7EDCD88EC1B}"/>
-    <hyperlink ref="A75" r:id="rId11" display="mailto:ozan.zeray@hotmail.com" xr:uid="{7B913CB5-A0DF-D244-BB40-392DE02F9CB1}"/>
-    <hyperlink ref="A76" r:id="rId12" display="mailto:karaserkan2@gmail.com" xr:uid="{FFF2B194-E361-5B4C-BA3A-83939AF0DA12}"/>
-    <hyperlink ref="A77" r:id="rId13" display="mailto:osmn.ozdmr.07@gmail.com" xr:uid="{A6775528-8948-2A43-9555-CA6DC1CDBCF4}"/>
-    <hyperlink ref="A78" r:id="rId14" display="mailto:radar1radar1org@gmail.com" xr:uid="{D6211F92-F75A-2A46-A7AC-D74E5729349F}"/>
-    <hyperlink ref="A79" r:id="rId15" display="mailto:tolga.yig@gmail.com" xr:uid="{2F9B8BC4-55E2-3143-88B3-1AF70CBDBAFC}"/>
-    <hyperlink ref="A80" r:id="rId16" display="mailto:akinturgut737@gmail.com" xr:uid="{C12E85A8-AAFC-BC4B-9A36-E112A50C1E3A}"/>
-    <hyperlink ref="A81" r:id="rId17" display="mailto:uakdemir@gmail.com" xr:uid="{2D5C8DA6-04EF-1845-95F5-1894BF31F43D}"/>
+    <hyperlink ref="A69" r:id="rId1" display="mailto:alperensarcayr@gmail.com" xr:uid="{06658918-687B-1347-B675-CC5C5BFCF91F}"/>
+    <hyperlink ref="A70" r:id="rId2" display="mailto:info@elchedo.pro" xr:uid="{F237D509-9129-BE47-A18D-473A1A06207A}"/>
+    <hyperlink ref="A71" r:id="rId3" display="mailto:cc5141864@gmail.com" xr:uid="{61FC5266-8368-DD4F-B177-452C3C0903D8}"/>
+    <hyperlink ref="A72" r:id="rId4" display="mailto:dguk21@gmail.com" xr:uid="{D68F8747-E451-934A-A817-A48D53F72BD5}"/>
+    <hyperlink ref="A73" r:id="rId5" display="mailto:capkurtdidemsevim@gmail.com" xr:uid="{B252AC13-D35C-D042-8AF8-0829EF8FBF9F}"/>
+    <hyperlink ref="A74" r:id="rId6" display="mailto:dogukanturksoy1999@gmail.com" xr:uid="{1E3D7200-4681-BE4D-9064-98D0E903E19C}"/>
+    <hyperlink ref="A75" r:id="rId7" display="mailto:eyuphantilki41@gmail.com" xr:uid="{5643087D-A516-DE4F-B3A1-ABD32096C308}"/>
+    <hyperlink ref="A76" r:id="rId8" display="mailto:kiymazaslanfatma@gmail.com" xr:uid="{39EF22EA-85E5-994E-A5CF-1BF1F5BBFD0F}"/>
+    <hyperlink ref="A77" r:id="rId9" display="mailto:Kirogluhasan08@gmail.com" xr:uid="{7720F11B-F4BF-9945-9159-503646E88A7E}"/>
+    <hyperlink ref="A78" r:id="rId10" display="mailto:bakicapica@gmail.com" xr:uid="{59A7D5F2-AB8E-054F-882C-D7EDCD88EC1B}"/>
+    <hyperlink ref="A79" r:id="rId11" display="mailto:ozan.zeray@hotmail.com" xr:uid="{7B913CB5-A0DF-D244-BB40-392DE02F9CB1}"/>
+    <hyperlink ref="A80" r:id="rId12" display="mailto:karaserkan2@gmail.com" xr:uid="{FFF2B194-E361-5B4C-BA3A-83939AF0DA12}"/>
+    <hyperlink ref="A81" r:id="rId13" display="mailto:osmn.ozdmr.07@gmail.com" xr:uid="{A6775528-8948-2A43-9555-CA6DC1CDBCF4}"/>
+    <hyperlink ref="A82" r:id="rId14" display="mailto:radar1radar1org@gmail.com" xr:uid="{D6211F92-F75A-2A46-A7AC-D74E5729349F}"/>
+    <hyperlink ref="A83" r:id="rId15" display="mailto:tolga.yig@gmail.com" xr:uid="{2F9B8BC4-55E2-3143-88B3-1AF70CBDBAFC}"/>
+    <hyperlink ref="A84" r:id="rId16" display="mailto:akinturgut737@gmail.com" xr:uid="{C12E85A8-AAFC-BC4B-9A36-E112A50C1E3A}"/>
+    <hyperlink ref="A85" r:id="rId17" display="mailto:uakdemir@gmail.com" xr:uid="{2D5C8DA6-04EF-1845-95F5-1894BF31F43D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>

</xml_diff>